<commit_message>
AllRegions value changed from 5 to 10
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_ElasticDem.xlsx
+++ b/SuppXLS/Scen_ElasticDem.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\Demo_models\DemoS_010\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16B28BB-84D4-4999-8F4A-8D67797A01D7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Elasticity_Data" sheetId="10" r:id="rId1"/>
+    <sheet name="Elasticity_Data" sheetId="10" r:id="rId3"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,106 +33,106 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="34">
   <si>
+    <t>UP</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
+  </si>
+  <si>
+    <t>DRAP,DROT</t>
+  </si>
+  <si>
+    <t>DRSH</t>
+  </si>
+  <si>
+    <t>LO</t>
+  </si>
+  <si>
+    <t>COM_ELAST</t>
+  </si>
+  <si>
+    <t>LO,UP</t>
+  </si>
+  <si>
+    <t>DCSH</t>
+  </si>
+  <si>
+    <t>Case Demos_007</t>
+  </si>
+  <si>
+    <t>DIDM1</t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>Figure 4</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>Case Demos_007a with CO2 bound</t>
+  </si>
+  <si>
+    <t>DAOT</t>
+  </si>
+  <si>
+    <t>Figure 5 GDX file selection for the elastic demand run</t>
+  </si>
+  <si>
+    <t>Case Demos_007b with CO2 bounds and elastic demand</t>
+  </si>
+  <si>
+    <t>UP,LO</t>
+  </si>
+  <si>
+    <t>Cset_CN</t>
+  </si>
+  <si>
+    <t>Cset_Set</t>
+  </si>
+  <si>
+    <t>AllRegions</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>DTCAR,DTPUB</t>
+  </si>
+  <si>
+    <t>* update values and insert new parameters for elastic demands (new scenario)</t>
+  </si>
+  <si>
+    <t>DCAP,DCOT</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>ANNUAL</t>
+  </si>
+  <si>
+    <t>2006,2050</t>
+  </si>
+  <si>
+    <t>COM_STEP</t>
+  </si>
+  <si>
+    <t>DEM</t>
+  </si>
+  <si>
+    <t>COM_VOC</t>
+  </si>
+  <si>
     <t>Attribute</t>
   </si>
   <si>
-    <t>LO</t>
-  </si>
-  <si>
-    <t>UP</t>
-  </si>
-  <si>
-    <t>TimeSlice</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>AllRegions</t>
-  </si>
-  <si>
     <t>~TFM_INS</t>
-  </si>
-  <si>
-    <t>ANNUAL</t>
-  </si>
-  <si>
-    <t>* update values and insert new parameters for elastic demands (new scenario)</t>
-  </si>
-  <si>
-    <t>COM_ELAST</t>
-  </si>
-  <si>
-    <t>COM_VOC</t>
-  </si>
-  <si>
-    <t>COM_STEP</t>
-  </si>
-  <si>
-    <t>UP,LO</t>
-  </si>
-  <si>
-    <t>Figure 1</t>
-  </si>
-  <si>
-    <t>Figure 2</t>
-  </si>
-  <si>
-    <t>Case Demos_007</t>
-  </si>
-  <si>
-    <t>Figure 3</t>
-  </si>
-  <si>
-    <t>Figure 4</t>
-  </si>
-  <si>
-    <t>Case Demos_007b with CO2 bounds and elastic demand</t>
-  </si>
-  <si>
-    <t>Case Demos_007a with CO2 bound</t>
-  </si>
-  <si>
-    <t>Figure 5 GDX file selection for the elastic demand run</t>
-  </si>
-  <si>
-    <t>Cset_Set</t>
-  </si>
-  <si>
-    <t>DEM</t>
-  </si>
-  <si>
-    <t>2006,2050</t>
-  </si>
-  <si>
-    <t>LO,UP</t>
-  </si>
-  <si>
-    <t>DTCAR,DTPUB</t>
-  </si>
-  <si>
-    <t>DRSH</t>
-  </si>
-  <si>
-    <t>DRAP,DROT</t>
-  </si>
-  <si>
-    <t>DCSH</t>
-  </si>
-  <si>
-    <t>DCAP,DCOT</t>
-  </si>
-  <si>
-    <t>DAOT</t>
-  </si>
-  <si>
-    <t>DIDM1</t>
   </si>
 </sst>
 </file>
@@ -142,13 +142,19 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -197,13 +203,6 @@
       <family val="3"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,12 +219,14 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -244,13 +245,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="44"/>
+        <fgColor rgb="FFFFFF99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
+        <fgColor indexed="44"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -267,92 +268,271 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom/>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="14">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
+  <cellStyleXfs count="33">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="22" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="22" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="22" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="13"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="13" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="13" applyFont="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="13" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="13" fillId="0" borderId="0" xfId="13" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="22" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="22" applyNumberFormat="1" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="22" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="22" applyFont="1" quotePrefix="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="22" applyFont="1" applyBorder="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="22" applyFont="1" applyBorder="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="32">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="32" applyNumberFormat="1" applyFont="1" quotePrefix="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="32" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="32" applyNumberFormat="1" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="32" applyNumberFormat="1" applyFont="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection/>
+    </xf>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" wrapText="1"/>
+      <protection/>
+    </xf>
   </cellXfs>
-  <cellStyles count="14">
-    <cellStyle name="Comma 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+  <cellStyles count="19">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 2 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Normal 4" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Normal 4 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Normal 5" xfId="13" xr:uid="{94A6A89F-51B7-4DB9-BFE6-BDFD2FF6CC7E}"/>
-    <cellStyle name="Normal 8" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="Normal 9 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Normale_B2020" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Percent 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="Standard_Sce_D_Extraction" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Percent" xfId="15" builtinId="5"/>
+    <cellStyle name="Currency" xfId="16" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
+    <cellStyle name="Comma" xfId="18" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
+    <cellStyle name="Comma 2" xfId="20"/>
+    <cellStyle name="Normal 10" xfId="21"/>
+    <cellStyle name="Normal 2" xfId="22"/>
+    <cellStyle name="Normal 2 2" xfId="23"/>
+    <cellStyle name="Normal 3" xfId="24"/>
+    <cellStyle name="Normal 4" xfId="25"/>
+    <cellStyle name="Normal 4 2" xfId="26"/>
+    <cellStyle name="Normal 8" xfId="27"/>
+    <cellStyle name="Normal 9 2" xfId="28"/>
+    <cellStyle name="Normale_B2020" xfId="29"/>
+    <cellStyle name="Percent 2" xfId="30"/>
+    <cellStyle name="Standard_Sce_D_Extraction" xfId="31"/>
+    <cellStyle name="Normal 5" xfId="32"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -365,7 +545,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
@@ -379,12 +559,12 @@
       <xdr:row>29</xdr:row>
       <xdr:rowOff>52916</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
+    <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14CB7748-959C-4BA0-9C7B-A640896FF2D1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14cb7748-959c-4ba0-9c7b-a640896ff2d1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -392,12 +572,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5828242" y="220130"/>
-          <a:ext cx="6025091" cy="5399619"/>
+          <a:off x="5800725" y="219075"/>
+          <a:ext cx="5991225" cy="5400675"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
         <a:solidFill>
           <a:schemeClr val="accent6">
             <a:lumMod val="20000"/>
@@ -406,7 +584,7 @@
         </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
-            <a:schemeClr val="lt1">
+            <a:schemeClr val="bg1">
               <a:shade val="50000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -414,16 +592,16 @@
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:lnRef>
         <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
+          <a:srgbClr val="000000"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
@@ -434,7 +612,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1600" b="1">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -448,7 +626,7 @@
           <a:pPr lvl="0"/>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -461,7 +639,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" b="1">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -473,7 +651,7 @@
           <a:r>
             <a:rPr lang="en-US" sz="1100" u="sng">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -483,15 +661,18 @@
             <a:t>Solve the reference case</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB" sz="1100" u="sng">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -503,7 +684,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -514,7 +695,7 @@
           </a:r>
           <a:endParaRPr lang="en-CA" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -523,11 +704,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -539,7 +720,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -551,7 +732,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -563,7 +744,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -576,7 +757,7 @@
         <a:p>
           <a:endParaRPr lang="en-CA" sz="1100" baseline="0">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -588,7 +769,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" b="1" i="1" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -601,7 +782,7 @@
         <a:p>
           <a:endParaRPr lang="en-CA" sz="1100" baseline="0">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -610,11 +791,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100" b="1" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -626,7 +807,7 @@
           <a:r>
             <a:rPr lang="en-US" sz="1100" u="sng">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -637,7 +818,7 @@
           </a:r>
           <a:endParaRPr lang="en-GB" sz="1100" u="sng">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -646,11 +827,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -660,15 +841,18 @@
             <a:t>- Including CO2 emission constraint or tax, etc</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -679,11 +863,11 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -694,11 +878,11 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -708,13 +892,16 @@
             <a:t>	COM_STEP: Number of steps to use for the approximation of change of 	producer/consumer surplus when using the elastic  demand formulation. (e.g. 10)</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -723,11 +910,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -739,7 +926,7 @@
           <a:r>
             <a:rPr lang="en-US" sz="1100" u="sng">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -750,7 +937,7 @@
           </a:r>
           <a:endParaRPr lang="en-GB" sz="1100" u="sng">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -759,11 +946,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -775,7 +962,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -785,15 +972,18 @@
             <a:t> for example DemoS_007a (Figure 3) include the two scenario ELC_CO2_BOUND and TRA_CO2_BOUND.</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -805,7 +995,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -817,7 +1007,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -828,7 +1018,7 @@
           </a:r>
           <a:endParaRPr lang="en-GB" sz="1100">
             <a:solidFill>
-              <a:schemeClr val="dk1"/>
+              <a:schemeClr val="tx1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="+mn-lt"/>
@@ -837,11 +1027,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-GB" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -853,7 +1043,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -865,7 +1055,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -877,7 +1067,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -889,7 +1079,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -899,15 +1089,18 @@
             <a:t>:</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -918,11 +1111,11 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -933,11 +1126,11 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -949,7 +1142,7 @@
           <a:r>
             <a:rPr lang="en-GB" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -961,7 +1154,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -973,7 +1166,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -985,7 +1178,7 @@
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -996,11 +1189,11 @@
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr rtl="0" eaLnBrk="1" fontAlgn="base" hangingPunct="1"/>
+          <a:pPr fontAlgn="base" hangingPunct="1" eaLnBrk="1" rtl="0"/>
           <a:r>
             <a:rPr lang="en-CA" sz="1100">
               <a:solidFill>
-                <a:schemeClr val="dk1"/>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="+mn-lt"/>
@@ -1010,6 +1203,9 @@
             <a:t>        - Run the case Demos_007b</a:t>
           </a:r>
           <a:endParaRPr lang="en-GB">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
@@ -1035,16 +1231,18 @@
         <xdr:cNvPr id="6" name="Group 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B7E0DB2-24CC-41D0-87AC-E4B07572401E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2b7e0db2-24cc-41d0-87ac-e4b07572401e}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
+        <xdr:cNvGrpSpPr>
+          <a:grpSpLocks/>
+        </xdr:cNvGrpSpPr>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="11938000" y="402168"/>
-          <a:ext cx="2733144" cy="4255462"/>
+          <a:off x="11868150" y="400050"/>
+          <a:ext cx="2714625" cy="4257675"/>
           <a:chOff x="11828318" y="398319"/>
           <a:chExt cx="2702357" cy="4251614"/>
         </a:xfrm>
@@ -1054,7 +1252,7 @@
           <xdr:cNvPr id="5" name="Picture 4">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6150CFAF-DF7D-4199-8CD3-6CD121B8C324}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6150cfaf-df7d-4199-8cd3-6cd121b8c324}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1063,7 +1261,7 @@
           </xdr:cNvPicPr>
         </xdr:nvPicPr>
         <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+          <a:blip r:embed="rId1"/>
           <a:stretch>
             <a:fillRect/>
           </a:stretch>
@@ -1073,17 +1271,15 @@
             <a:off x="11828318" y="398319"/>
             <a:ext cx="2702357" cy="4251614"/>
           </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
+          <a:prstGeom prst="rect"/>
         </xdr:spPr>
       </xdr:pic>
-      <xdr:sp macro="" textlink="">
+      <xdr:sp>
         <xdr:nvSpPr>
           <xdr:cNvPr id="4" name="Oval 3">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F67A5C16-3E73-4E92-81E5-9DD6C28D2231}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{f67a5c16-3e73-4e92-81e5-9dd6c28d2231}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1094,9 +1290,7 @@
             <a:off x="11914909" y="4372841"/>
             <a:ext cx="1743075" cy="268432"/>
           </a:xfrm>
-          <a:prstGeom prst="ellipse">
-            <a:avLst/>
-          </a:prstGeom>
+          <a:prstGeom prst="ellipse"/>
           <a:noFill/>
           <a:ln>
             <a:solidFill>
@@ -1117,7 +1311,7 @@
             <a:schemeClr val="accent1"/>
           </a:effectRef>
           <a:fontRef idx="minor">
-            <a:schemeClr val="lt1"/>
+            <a:schemeClr val="bg1"/>
           </a:fontRef>
         </xdr:style>
         <xdr:txBody>
@@ -1141,15 +1335,15 @@
     <xdr:to>
       <xdr:col>29</xdr:col>
       <xdr:colOff>192559</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>181842</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{358DB482-7514-49DF-9A37-62BF3644A258}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{358db482-7514-49df-9a37-62bf3644a258}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1158,19 +1352,17 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14848249" y="406978"/>
-          <a:ext cx="3233992" cy="3619500"/>
+          <a:off x="14906625" y="409575"/>
+          <a:ext cx="3257550" cy="3629025"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1193,7 +1385,7 @@
         <xdr:cNvPr id="8" name="Picture 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{716E77ED-0E02-4676-BBD7-0B35BA239866}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{716e77ed-0e02-4676-bbd7-0b35ba239866}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1202,19 +1394,17 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5842001" y="5408083"/>
-          <a:ext cx="7087266" cy="3180750"/>
+          <a:off x="5810250" y="5972175"/>
+          <a:ext cx="7038975" cy="3181350"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1237,16 +1427,18 @@
         <xdr:cNvPr id="12" name="Group 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9641BA90-B21C-4D8F-9F5C-B8406F007226}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9641ba90-b21c-4d8f-9f5c-b8406f007226}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
+        <xdr:cNvGrpSpPr>
+          <a:grpSpLocks/>
+        </xdr:cNvGrpSpPr>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13155084" y="5965122"/>
-          <a:ext cx="7155658" cy="3200045"/>
+          <a:off x="13077825" y="5962650"/>
+          <a:ext cx="7105650" cy="3200400"/>
           <a:chOff x="13155084" y="5584122"/>
           <a:chExt cx="7155658" cy="3200045"/>
         </a:xfrm>
@@ -1256,7 +1448,7 @@
           <xdr:cNvPr id="11" name="Picture 10">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E89CFAF-BA5B-4CC4-B235-6744C879781B}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8e89cfaf-ba5b-4cc4-b235-6744c879781b}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1265,7 +1457,7 @@
           </xdr:cNvPicPr>
         </xdr:nvPicPr>
         <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+          <a:blip r:embed="rId4"/>
           <a:stretch>
             <a:fillRect/>
           </a:stretch>
@@ -1275,17 +1467,15 @@
             <a:off x="13155084" y="5584122"/>
             <a:ext cx="7155658" cy="3200045"/>
           </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
+          <a:prstGeom prst="rect"/>
         </xdr:spPr>
       </xdr:pic>
-      <xdr:sp macro="" textlink="">
+      <xdr:sp>
         <xdr:nvSpPr>
           <xdr:cNvPr id="10" name="Oval 9">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7D07189-3274-4673-9C9F-26B855F1333F}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{c7d07189-3274-4673-9c9f-26b855f1333f}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1296,9 +1486,7 @@
             <a:off x="17430750" y="8244417"/>
             <a:ext cx="1513417" cy="349250"/>
           </a:xfrm>
-          <a:prstGeom prst="ellipse">
-            <a:avLst/>
-          </a:prstGeom>
+          <a:prstGeom prst="ellipse"/>
           <a:noFill/>
           <a:ln>
             <a:solidFill>
@@ -1319,7 +1507,7 @@
             <a:schemeClr val="accent1"/>
           </a:effectRef>
           <a:fontRef idx="minor">
-            <a:schemeClr val="lt1"/>
+            <a:schemeClr val="bg1"/>
           </a:fontRef>
         </xdr:style>
         <xdr:txBody>
@@ -1352,7 +1540,7 @@
         <xdr:cNvPr id="13" name="Picture 12">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{298A4DBC-AF3E-4130-9EB3-2EF369B271B2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{298a4dbc-af3e-4130-9eb3-2ef369b271b2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1361,19 +1549,17 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:blip r:embed="rId5"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="20531668" y="5566834"/>
-          <a:ext cx="3518222" cy="3206750"/>
+          <a:off x="20402550" y="5943600"/>
+          <a:ext cx="3495675" cy="3209925"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1701,37 +1887,37 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:AH41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" customWidth="1"/>
-    <col min="2" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.42857142857143" customWidth="1"/>
+    <col min="2" max="3" width="8.85714285714286" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1428571428571" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15.75">
       <c r="A1" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" ht="15.75">
       <c r="A2" s="1"/>
       <c r="T2" s="10" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="Y2" s="10" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="Z2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="15">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1752,10 +1938,10 @@
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="15">
       <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -1775,28 +1961,28 @@
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
     </row>
-    <row r="5" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" ht="15.75" thickBot="1">
       <c r="A5" s="2"/>
       <c r="B5" s="5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -1810,20 +1996,20 @@
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="15">
       <c r="A6" s="2"/>
       <c r="B6" s="11"/>
       <c r="C6" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E6" s="4">
         <v>2006</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4">
@@ -1841,19 +2027,19 @@
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="15">
       <c r="A7" s="2"/>
       <c r="C7" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E7" s="4">
         <v>2030</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4">
@@ -1871,24 +2057,24 @@
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="15">
       <c r="A8" s="2"/>
       <c r="B8" s="11"/>
       <c r="C8" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E8" s="4">
         <v>2050</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="12">
-        <v>0.3</v>
+        <v>0.30</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -1902,20 +2088,20 @@
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="15">
       <c r="A9" s="2"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="E9" s="4">
         <v>0</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4">
@@ -1933,20 +2119,20 @@
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="15">
       <c r="A10" s="7"/>
       <c r="B10" s="13"/>
       <c r="C10" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4">
@@ -1964,12 +2150,12 @@
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="15">
       <c r="A11" s="2"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" ht="15">
       <c r="B13" s="3" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -1978,595 +2164,595 @@
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="15.75" thickBot="1">
       <c r="B14" s="8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" ht="15">
+      <c r="B15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="E15" s="4">
         <v>2006</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" s="12">
+        <v>-0.033000000000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" ht="15">
+      <c r="B16" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H15" s="12">
-        <v>-3.3000000000000002E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="C16" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E16" s="4">
         <v>2015</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H16" s="4">
         <v>-0.15</v>
       </c>
     </row>
-    <row r="17" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" ht="15">
       <c r="B17" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E17" s="4">
         <v>2015</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H17" s="4">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="18" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:8" ht="15">
       <c r="B18" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E18" s="4">
         <v>2030</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" s="12">
+        <v>-0.30</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="15">
+      <c r="B19" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="H18" s="12">
-        <v>-0.3</v>
-      </c>
-    </row>
-    <row r="19" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="B19" s="15" t="s">
-        <v>9</v>
-      </c>
       <c r="C19" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E19" s="15">
         <v>2030</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H19" s="15">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="20" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:8" ht="15">
       <c r="B20" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E20" s="4">
         <v>2006</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="H20" s="12">
         <v>-0.03</v>
       </c>
     </row>
-    <row r="21" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:8" ht="15">
       <c r="B21" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E21" s="4">
         <v>2015</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="H21" s="12">
-        <v>-0.5</v>
-      </c>
-    </row>
-    <row r="22" spans="2:34" x14ac:dyDescent="0.25">
+        <v>-0.50</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="15">
       <c r="B22" s="15" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E22" s="15">
         <v>2015</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="H22" s="15">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="23" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:8" ht="15">
       <c r="B23" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E23" s="4">
         <v>2006</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="H23" s="12">
-        <v>-3.3000000000000002E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="2:34" x14ac:dyDescent="0.25">
+        <v>-0.033000000000000002</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="15">
       <c r="B24" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E24" s="4">
         <v>2015</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="H24" s="12">
-        <v>-0.3</v>
-      </c>
-    </row>
-    <row r="25" spans="2:34" x14ac:dyDescent="0.25">
+        <v>-0.30</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="15">
       <c r="B25" s="15" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E25" s="15">
         <v>2015</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="H25" s="15">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="26" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:8" ht="15">
       <c r="B26" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E26" s="4">
         <v>2006</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="H26" s="12">
         <v>-0.03</v>
       </c>
     </row>
-    <row r="27" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:8" ht="15">
       <c r="B27" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E27" s="4">
         <v>2015</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="H27" s="12">
-        <v>-0.5</v>
-      </c>
-    </row>
-    <row r="28" spans="2:34" x14ac:dyDescent="0.25">
+        <v>-0.50</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" ht="15">
       <c r="B28" s="15" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E28" s="15">
         <v>2015</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="H28" s="15">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="29" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:8" ht="15">
       <c r="B29" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E29" s="4">
         <v>2006</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="H29" s="12">
-        <v>-3.3000000000000002E-2</v>
-      </c>
-    </row>
-    <row r="30" spans="2:34" x14ac:dyDescent="0.25">
+        <v>-0.033000000000000002</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" ht="15">
       <c r="B30" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E30" s="4">
         <v>2015</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="H30" s="12">
-        <v>-0.3</v>
-      </c>
-    </row>
-    <row r="31" spans="2:34" x14ac:dyDescent="0.25">
+        <v>-0.30</v>
+      </c>
+    </row>
+    <row r="31" spans="2:34" ht="15">
       <c r="B31" s="15" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E31" s="15">
         <v>2015</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="H31" s="15">
         <v>-0.05</v>
       </c>
       <c r="J31" s="10" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K31" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="V31" s="10" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="W31" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AH31" s="10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="2:34" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" ht="15">
       <c r="B32" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E32" s="4">
         <v>2006</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="H32" s="12">
         <v>-0.03</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:8" ht="15">
       <c r="B33" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E33" s="4">
         <v>2015</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="H33" s="12">
-        <v>-0.3</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+        <v>-0.30</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" ht="15">
       <c r="B34" s="15" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E34" s="15">
         <v>2015</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="H34" s="15">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:8" ht="15">
       <c r="B35" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E35" s="4">
         <v>2006</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H35" s="12">
         <v>-0.03</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:8" ht="15">
       <c r="B36" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E36" s="4">
         <v>2015</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H36" s="12">
-        <v>-0.3</v>
-      </c>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+        <v>-0.30</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" ht="15">
       <c r="B37" s="15" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E37" s="15">
         <v>2015</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H37" s="15">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B38" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" s="4">
+    <row r="38" spans="2:8" ht="15">
+      <c r="B38" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="E38" s="23">
         <v>0</v>
       </c>
-      <c r="F38" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G38" s="4"/>
-      <c r="H38" s="12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F38" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="G38" s="22"/>
+      <c r="H38" s="24">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" ht="15">
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
@@ -2575,7 +2761,7 @@
       <c r="G39" s="20"/>
       <c r="H39" s="21"/>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:8" ht="15">
       <c r="B40" s="17"/>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -2584,7 +2770,7 @@
       <c r="G40" s="20"/>
       <c r="H40" s="21"/>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:8" ht="15">
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
       <c r="D41" s="17"/>
@@ -2594,9 +2780,8 @@
       <c r="H41" s="21"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup orientation="portrait" paperSize="1" r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>